<commit_message>
style: standardize fonts in Excel file
</commit_message>
<xml_diff>
--- a/시도별_통합데이터_2024.xlsx
+++ b/시도별_통합데이터_2024.xlsx
@@ -1,16 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rose0\OneDrive\Desktop\2026\대학교\2학기\공모전\AI와 함께하는 교통문제 해결을 위한 데이터 분석 공모전\kpass-regional-gap\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32AE5939-DD29-44CF-82CF-2B70DE17473C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="450" yWindow="600" windowWidth="24640" windowHeight="13680"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="통합데이터" sheetId="1" r:id="rId1"/>
     <sheet name="비용계산근거" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -20,1498 +39,479 @@
     <t>시도명</t>
   </si>
   <si>
+    <t>용도별_차종별_시군구별_자동차주행거리(KOSIS 국가통계포털)_2024_비사업용_승용차_연간 주행거리(천㎞)</t>
+  </si>
+  <si>
+    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_일반_이용인원(명)</t>
+  </si>
+  <si>
+    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_어린이_이용인원(명)</t>
+  </si>
+  <si>
+    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_청소년_이용인원(명)</t>
+  </si>
+  <si>
+    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_고령자_이용인원(명)</t>
+  </si>
+  <si>
+    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_기타_이용인원(명)</t>
+  </si>
+  <si>
+    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_월_이용인원</t>
+  </si>
+  <si>
+    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_화_이용인원</t>
+  </si>
+  <si>
+    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_수_이용인원</t>
+  </si>
+  <si>
+    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_목_이용인원</t>
+  </si>
+  <si>
+    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_금_이용인원</t>
+  </si>
+  <si>
+    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_토_이용인원</t>
+  </si>
+  <si>
+    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_일_이용인원</t>
+  </si>
+  <si>
+    <t>자동차등록대수현황_시도별(2024.12)_2024.12_승용_자가용(대)</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_0세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_1세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_2세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_3세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_4세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_5세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_6세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_7세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_8세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_9세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_10세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_11세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_12세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_13세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_14세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_15세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_16세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_17세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_18세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_19세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_20세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_21세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_22세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_23세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_24세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_25세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_26세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_27세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_28세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_29세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_30세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_31세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_32세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_33세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_34세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_35세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_36세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_37세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_38세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_39세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_40세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_41세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_42세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_43세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_44세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_45세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_46세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_47세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_48세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_49세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_50세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_51세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_52세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_53세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_54세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_55세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_56세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_57세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_58세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_59세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_60세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_61세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_62세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_63세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_64세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_65세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_66세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_67세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_68세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_69세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_70세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_71세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_72세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_73세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_74세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_75세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_76세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_77세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_78세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_79세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_80세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_81세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_82세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_83세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_84세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_85세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_86세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_87세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_88세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_89세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_90세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_91세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_92세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_93세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_94세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_95세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_96세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_97세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_98세</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_99세</t>
+  </si>
+  <si>
+    <t>서울특별시</t>
+  </si>
+  <si>
+    <t>부산광역시</t>
+  </si>
+  <si>
+    <t>대구광역시</t>
+  </si>
+  <si>
+    <t>인천광역시</t>
+  </si>
+  <si>
+    <t>광주광역시</t>
+  </si>
+  <si>
+    <t>대전광역시</t>
+  </si>
+  <si>
+    <t>울산광역시</t>
+  </si>
+  <si>
+    <t>세종특별자치시</t>
+  </si>
+  <si>
+    <t>경기도</t>
+  </si>
+  <si>
+    <t>강원특별자치도</t>
+  </si>
+  <si>
+    <t>충청북도</t>
+  </si>
+  <si>
+    <t>충청남도</t>
+  </si>
+  <si>
+    <t>전북특별자치도</t>
+  </si>
+  <si>
+    <t>전라남도</t>
+  </si>
+  <si>
+    <t>경상북도</t>
+  </si>
+  <si>
+    <t>경상남도</t>
+  </si>
+  <si>
+    <t>제주특별자치도</t>
+  </si>
+  <si>
+    <t>2만원 미만</t>
+  </si>
+  <si>
+    <t>2만원~4만원</t>
+  </si>
+  <si>
+    <t>4만원~6만원</t>
+  </si>
+  <si>
+    <t>6만원~8만원</t>
+  </si>
+  <si>
+    <t>8만원~10만원</t>
+  </si>
+  <si>
+    <t>10만원~12만원</t>
+  </si>
+  <si>
+    <t>12만원 이상</t>
+  </si>
+  <si>
+    <t>원본 비율 합계(%)</t>
+  </si>
+  <si>
+    <t>월평균 비용(만원)</t>
+  </si>
+  <si>
+    <t>구간 대표값(만원)</t>
+  </si>
+  <si>
+    <t>계산 방식: 원본 비율 × 구간 대표값의 합 ÷ 100. 비율 합계 보정 없음.</t>
+  </si>
+  <si>
+    <t>출처: 시도별_월평균_대중교통비용(KOSIS 국가통계포털)(1).xlsx / 데이터 시트 / 2024년 / 원본 단위 %</t>
+  </si>
+  <si>
+    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_100세 이상</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>배차간격_요일별(TS 한국교통안전공단)_2024_월_배차간격(분)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>배차간격_요일별(TS 한국교통안전공단)_2024_화_배차간격(분)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>배차간격_요일별(TS 한국교통안전공단)_2024_수_배차간격(분)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>배차간격_요일별(TS 한국교통안전공단)_2024_목_배차간격(분)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>배차간격_요일별(TS 한국교통안전공단)_2024_금_배차간격(분)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>배차간격_요일별(TS 한국교통안전공단)_2024_토_배차간격(분)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>배차간격_요일별(TS 한국교통안전공단)_2024_일_배차간격(분)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>시도별_월평균_대중교통비용(KOSIS 국가통계포털)(1)_2024_월평균 비용(만원)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
     <t>용도별_차종별_시군구별_자동차주행거리(KOSIS 국가통계포털)_2024_비사업용_승용차_1일 평균주행거리(㎞/대)</t>
-  </si>
-  <si>
-    <t>용도별_차종별_시군구별_자동차주행거리(KOSIS 국가통계포털)_2024_비사업용_승용차_연간 주행거리(천㎞)</t>
-  </si>
-  <si>
-    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_일반_이용인원(명)</t>
-  </si>
-  <si>
-    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_어린이_이용인원(명)</t>
-  </si>
-  <si>
-    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_청소년_이용인원(명)</t>
-  </si>
-  <si>
-    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_고령자_이용인원(명)</t>
-  </si>
-  <si>
-    <t>유형별 총 이용인원(TS 한국교통안전공단)_2024_기타_이용인원(명)</t>
-  </si>
-  <si>
-    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_월_이용인원</t>
-  </si>
-  <si>
-    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_화_이용인원</t>
-  </si>
-  <si>
-    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_수_이용인원</t>
-  </si>
-  <si>
-    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_목_이용인원</t>
-  </si>
-  <si>
-    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_금_이용인원</t>
-  </si>
-  <si>
-    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_토_이용인원</t>
-  </si>
-  <si>
-    <t>시도별 총 이용인원(TS 한국교통안전공단)_2024_일_이용인원</t>
-  </si>
-  <si>
-    <t>자동차등록대수현황_시도별(2024.12)_2024.12_승용_자가용(대)</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_0세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_1세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_2세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_3세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_4세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_5세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_6세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_7세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_8세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_9세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_10세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_11세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_12세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_13세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_14세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_15세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_16세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_17세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_18세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_19세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_20세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_21세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_22세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_23세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_24세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_25세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_26세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_27세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_28세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_29세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_30세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_31세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_32세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_33세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_34세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_35세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_36세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_37세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_38세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_39세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_40세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_41세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_42세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_43세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_44세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_45세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_46세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_47세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_48세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_49세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_50세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_51세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_52세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_53세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_54세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_55세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_56세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_57세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_58세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_59세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_60세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_61세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_62세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_63세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_64세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_65세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_66세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_67세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_68세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_69세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_70세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_71세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_72세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_73세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_74세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_75세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_76세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_77세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_78세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_79세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_80세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_81세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_82세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_83세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_84세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_85세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_86세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_87세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_88세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_89세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_90세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_91세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_92세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_93세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_94세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_95세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_96세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_97세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_98세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_99세</t>
-  </si>
-  <si>
-    <t>행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_100세 이상</t>
-  </si>
-  <si>
-    <t>서울특별시</t>
-  </si>
-  <si>
-    <t>부산광역시</t>
-  </si>
-  <si>
-    <t>대구광역시</t>
-  </si>
-  <si>
-    <t>인천광역시</t>
-  </si>
-  <si>
-    <t>광주광역시</t>
-  </si>
-  <si>
-    <t>대전광역시</t>
-  </si>
-  <si>
-    <t>울산광역시</t>
-  </si>
-  <si>
-    <t>세종특별자치시</t>
-  </si>
-  <si>
-    <t>경기도</t>
-  </si>
-  <si>
-    <t>강원특별자치도</t>
-  </si>
-  <si>
-    <t>충청북도</t>
-  </si>
-  <si>
-    <t>충청남도</t>
-  </si>
-  <si>
-    <t>전북특별자치도</t>
-  </si>
-  <si>
-    <t>전라남도</t>
-  </si>
-  <si>
-    <t>경상북도</t>
-  </si>
-  <si>
-    <t>경상남도</t>
-  </si>
-  <si>
-    <t>제주특별자치도</t>
-  </si>
-  <si>
-    <t>2만원 미만</t>
-  </si>
-  <si>
-    <t>2만원~4만원</t>
-  </si>
-  <si>
-    <t>4만원~6만원</t>
-  </si>
-  <si>
-    <t>6만원~8만원</t>
-  </si>
-  <si>
-    <t>8만원~10만원</t>
-  </si>
-  <si>
-    <t>10만원~12만원</t>
-  </si>
-  <si>
-    <t>12만원 이상</t>
-  </si>
-  <si>
-    <t>원본 비율 합계(%)</t>
-  </si>
-  <si>
-    <t>월평균 비용(만원)</t>
-  </si>
-  <si>
-    <t>구간 대표값(만원)</t>
-  </si>
-  <si>
-    <t>계산 방식: 원본 비율 × 구간 대표값의 합 ÷ 100. 비율 합계 보정 없음.</t>
-  </si>
-  <si>
-    <t>출처: 시도별_월평균_대중교통비용(KOSIS 국가통계포털)(1).xlsx / 데이터 시트 / 2024년 / 원본 단위 %</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>요일별</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(TS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한국교통안전공단</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)_2024_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>월</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>분</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>요일별</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(TS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한국교통안전공단</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)_2024_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>화</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>분</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>요일별</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(TS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한국교통안전공단</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)_2024_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>수</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>분</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>요일별</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(TS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한국교통안전공단</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)_2024_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>일</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>분</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>요일별</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(TS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한국교통안전공단</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)_2024_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>토</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>분</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>요일별</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(TS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한국교통안전공단</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)_2024_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>금</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>분</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>요일별</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(TS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한국교통안전공단</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)_2024_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>목</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>배차간격</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>분</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>시도별</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>월평균</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>대중교통비용</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(KOSIS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>국가통계포털</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)(1)_2024_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>월평균</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>비용</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>만원</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="176" formatCode="#,##0.0"/>
     <numFmt numFmtId="177" formatCode="0.0"/>
@@ -1548,7 +548,7 @@
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="돋움"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
     </font>
@@ -1589,62 +589,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="1"/>
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="124">
+  <dxfs count="125">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2023,138 +1041,141 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MergedData" displayName="MergedData" ref="A1:DU18" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MergedData" displayName="MergedData" ref="A1:DU18" totalsRowShown="0" headerRowDxfId="0">
   <tableColumns count="125">
-    <tableColumn id="1" name="시도명"/>
-    <tableColumn id="2" name="용도별_차종별_시군구별_자동차주행거리(KOSIS 국가통계포털)_2024_비사업용_승용차_1일 평균주행거리(㎞/대)" dataDxfId="123"/>
-    <tableColumn id="3" name="용도별_차종별_시군구별_자동차주행거리(KOSIS 국가통계포털)_2024_비사업용_승용차_연간 주행거리(천㎞)" dataDxfId="122"/>
-    <tableColumn id="4" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_일반_이용인원(명)" dataDxfId="121"/>
-    <tableColumn id="5" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_어린이_이용인원(명)" dataDxfId="120"/>
-    <tableColumn id="6" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_청소년_이용인원(명)" dataDxfId="119"/>
-    <tableColumn id="7" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_고령자_이용인원(명)" dataDxfId="118"/>
-    <tableColumn id="8" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_기타_이용인원(명)" dataDxfId="117"/>
-    <tableColumn id="9" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_월_이용인원" dataDxfId="116"/>
-    <tableColumn id="10" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_화_이용인원" dataDxfId="115"/>
-    <tableColumn id="11" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_수_이용인원" dataDxfId="114"/>
-    <tableColumn id="12" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_목_이용인원" dataDxfId="113"/>
-    <tableColumn id="13" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_금_이용인원" dataDxfId="112"/>
-    <tableColumn id="14" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_토_이용인원" dataDxfId="111"/>
-    <tableColumn id="15" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_일_이용인원" dataDxfId="110"/>
-    <tableColumn id="16" name="자동차등록대수현황_시도별(2024.12)_2024.12_승용_자가용(대)" dataDxfId="109"/>
-    <tableColumn id="17" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_0세" dataDxfId="108"/>
-    <tableColumn id="18" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_1세" dataDxfId="107"/>
-    <tableColumn id="19" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_2세" dataDxfId="106"/>
-    <tableColumn id="20" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_3세" dataDxfId="105"/>
-    <tableColumn id="21" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_4세" dataDxfId="104"/>
-    <tableColumn id="22" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_5세" dataDxfId="103"/>
-    <tableColumn id="23" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_6세" dataDxfId="102"/>
-    <tableColumn id="24" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_7세" dataDxfId="101"/>
-    <tableColumn id="25" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_8세" dataDxfId="100"/>
-    <tableColumn id="26" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_9세" dataDxfId="99"/>
-    <tableColumn id="27" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_10세" dataDxfId="98"/>
-    <tableColumn id="28" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_11세" dataDxfId="97"/>
-    <tableColumn id="29" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_12세" dataDxfId="96"/>
-    <tableColumn id="30" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_13세" dataDxfId="95"/>
-    <tableColumn id="31" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_14세" dataDxfId="94"/>
-    <tableColumn id="32" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_15세" dataDxfId="93"/>
-    <tableColumn id="33" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_16세" dataDxfId="92"/>
-    <tableColumn id="34" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_17세" dataDxfId="91"/>
-    <tableColumn id="35" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_18세" dataDxfId="90"/>
-    <tableColumn id="36" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_19세" dataDxfId="89"/>
-    <tableColumn id="37" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_20세" dataDxfId="88"/>
-    <tableColumn id="38" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_21세" dataDxfId="87"/>
-    <tableColumn id="39" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_22세" dataDxfId="86"/>
-    <tableColumn id="40" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_23세" dataDxfId="85"/>
-    <tableColumn id="41" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_24세" dataDxfId="84"/>
-    <tableColumn id="42" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_25세" dataDxfId="83"/>
-    <tableColumn id="43" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_26세" dataDxfId="82"/>
-    <tableColumn id="44" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_27세" dataDxfId="81"/>
-    <tableColumn id="45" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_28세" dataDxfId="80"/>
-    <tableColumn id="46" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_29세" dataDxfId="79"/>
-    <tableColumn id="47" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_30세" dataDxfId="78"/>
-    <tableColumn id="48" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_31세" dataDxfId="77"/>
-    <tableColumn id="49" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_32세" dataDxfId="76"/>
-    <tableColumn id="50" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_33세" dataDxfId="75"/>
-    <tableColumn id="51" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_34세" dataDxfId="74"/>
-    <tableColumn id="52" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_35세" dataDxfId="73"/>
-    <tableColumn id="53" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_36세" dataDxfId="72"/>
-    <tableColumn id="54" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_37세" dataDxfId="71"/>
-    <tableColumn id="55" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_38세" dataDxfId="70"/>
-    <tableColumn id="56" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_39세" dataDxfId="69"/>
-    <tableColumn id="57" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_40세" dataDxfId="68"/>
-    <tableColumn id="58" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_41세" dataDxfId="67"/>
-    <tableColumn id="59" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_42세" dataDxfId="66"/>
-    <tableColumn id="60" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_43세" dataDxfId="65"/>
-    <tableColumn id="61" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_44세" dataDxfId="64"/>
-    <tableColumn id="62" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_45세" dataDxfId="63"/>
-    <tableColumn id="63" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_46세" dataDxfId="62"/>
-    <tableColumn id="64" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_47세" dataDxfId="61"/>
-    <tableColumn id="65" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_48세" dataDxfId="60"/>
-    <tableColumn id="66" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_49세" dataDxfId="59"/>
-    <tableColumn id="67" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_50세" dataDxfId="58"/>
-    <tableColumn id="68" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_51세" dataDxfId="57"/>
-    <tableColumn id="69" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_52세" dataDxfId="56"/>
-    <tableColumn id="70" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_53세" dataDxfId="55"/>
-    <tableColumn id="71" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_54세" dataDxfId="54"/>
-    <tableColumn id="72" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_55세" dataDxfId="53"/>
-    <tableColumn id="73" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_56세" dataDxfId="52"/>
-    <tableColumn id="74" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_57세" dataDxfId="51"/>
-    <tableColumn id="75" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_58세" dataDxfId="50"/>
-    <tableColumn id="76" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_59세" dataDxfId="49"/>
-    <tableColumn id="77" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_60세" dataDxfId="48"/>
-    <tableColumn id="78" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_61세" dataDxfId="47"/>
-    <tableColumn id="79" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_62세" dataDxfId="46"/>
-    <tableColumn id="80" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_63세" dataDxfId="45"/>
-    <tableColumn id="81" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_64세" dataDxfId="44"/>
-    <tableColumn id="82" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_65세" dataDxfId="43"/>
-    <tableColumn id="83" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_66세" dataDxfId="42"/>
-    <tableColumn id="84" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_67세" dataDxfId="41"/>
-    <tableColumn id="85" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_68세" dataDxfId="40"/>
-    <tableColumn id="86" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_69세" dataDxfId="39"/>
-    <tableColumn id="87" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_70세" dataDxfId="38"/>
-    <tableColumn id="88" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_71세" dataDxfId="37"/>
-    <tableColumn id="89" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_72세" dataDxfId="36"/>
-    <tableColumn id="90" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_73세" dataDxfId="35"/>
-    <tableColumn id="91" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_74세" dataDxfId="34"/>
-    <tableColumn id="92" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_75세" dataDxfId="33"/>
-    <tableColumn id="93" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_76세" dataDxfId="32"/>
-    <tableColumn id="94" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_77세" dataDxfId="31"/>
-    <tableColumn id="95" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_78세" dataDxfId="30"/>
-    <tableColumn id="96" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_79세" dataDxfId="29"/>
-    <tableColumn id="97" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_80세" dataDxfId="28"/>
-    <tableColumn id="98" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_81세" dataDxfId="27"/>
-    <tableColumn id="99" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_82세" dataDxfId="26"/>
-    <tableColumn id="100" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_83세" dataDxfId="25"/>
-    <tableColumn id="101" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_84세" dataDxfId="24"/>
-    <tableColumn id="102" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_85세" dataDxfId="23"/>
-    <tableColumn id="103" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_86세" dataDxfId="22"/>
-    <tableColumn id="104" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_87세" dataDxfId="21"/>
-    <tableColumn id="105" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_88세" dataDxfId="20"/>
-    <tableColumn id="106" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_89세" dataDxfId="19"/>
-    <tableColumn id="107" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_90세" dataDxfId="18"/>
-    <tableColumn id="108" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_91세" dataDxfId="17"/>
-    <tableColumn id="109" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_92세" dataDxfId="16"/>
-    <tableColumn id="110" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_93세" dataDxfId="15"/>
-    <tableColumn id="111" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_94세" dataDxfId="14"/>
-    <tableColumn id="112" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_95세" dataDxfId="13"/>
-    <tableColumn id="113" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_96세" dataDxfId="12"/>
-    <tableColumn id="114" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_97세" dataDxfId="11"/>
-    <tableColumn id="115" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_98세" dataDxfId="10"/>
-    <tableColumn id="116" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_99세" dataDxfId="9"/>
-    <tableColumn id="117" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_100세 이상" dataDxfId="8"/>
-    <tableColumn id="118" name="배차간격_요일별(TS 한국교통안전공단)_2024_월_배차간격(분)" dataDxfId="7"/>
-    <tableColumn id="119" name="배차간격_요일별(TS 한국교통안전공단)_2024_화_배차간격(분)" dataDxfId="6"/>
-    <tableColumn id="120" name="배차간격_요일별(TS 한국교통안전공단)_2024_수_배차간격(분)" dataDxfId="5"/>
-    <tableColumn id="121" name="배차간격_요일별(TS 한국교통안전공단)_2024_목_배차간격(분)" dataDxfId="4"/>
-    <tableColumn id="122" name="배차간격_요일별(TS 한국교통안전공단)_2024_금_배차간격(분)" dataDxfId="3"/>
-    <tableColumn id="123" name="배차간격_요일별(TS 한국교통안전공단)_2024_토_배차간격(분)" dataDxfId="2"/>
-    <tableColumn id="124" name="배차간격_요일별(TS 한국교통안전공단)_2024_일_배차간격(분)" dataDxfId="1"/>
-    <tableColumn id="125" name="시도별_월평균_대중교통비용(KOSIS 국가통계포털)(1)_2024_월평균 비용(만원)" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="시도명"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="용도별_차종별_시군구별_자동차주행거리(KOSIS 국가통계포털)_2024_비사업용_승용차_1일 평균주행거리(㎞/대)" dataDxfId="124"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="용도별_차종별_시군구별_자동차주행거리(KOSIS 국가통계포털)_2024_비사업용_승용차_연간 주행거리(천㎞)" dataDxfId="123"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_일반_이용인원(명)" dataDxfId="122"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_어린이_이용인원(명)" dataDxfId="121"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_청소년_이용인원(명)" dataDxfId="120"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_고령자_이용인원(명)" dataDxfId="119"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="유형별 총 이용인원(TS 한국교통안전공단)_2024_기타_이용인원(명)" dataDxfId="118"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_월_이용인원" dataDxfId="117"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_화_이용인원" dataDxfId="116"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_수_이용인원" dataDxfId="115"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_목_이용인원" dataDxfId="114"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_금_이용인원" dataDxfId="113"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_토_이용인원" dataDxfId="112"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="시도별 총 이용인원(TS 한국교통안전공단)_2024_일_이용인원" dataDxfId="111"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="자동차등록대수현황_시도별(2024.12)_2024.12_승용_자가용(대)" dataDxfId="110"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_0세" dataDxfId="109"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_1세" dataDxfId="108"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_2세" dataDxfId="107"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_3세" dataDxfId="106"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_4세" dataDxfId="105"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_5세" dataDxfId="104"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_6세" dataDxfId="103"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_7세" dataDxfId="102"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_8세" dataDxfId="101"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_9세" dataDxfId="100"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_10세" dataDxfId="99"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_11세" dataDxfId="98"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_12세" dataDxfId="97"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_13세" dataDxfId="96"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_14세" dataDxfId="95"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_15세" dataDxfId="94"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_16세" dataDxfId="93"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_17세" dataDxfId="92"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_18세" dataDxfId="91"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_19세" dataDxfId="90"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_20세" dataDxfId="89"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_21세" dataDxfId="88"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_22세" dataDxfId="87"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_23세" dataDxfId="86"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_24세" dataDxfId="85"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_25세" dataDxfId="84"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_26세" dataDxfId="83"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_27세" dataDxfId="82"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_28세" dataDxfId="81"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_29세" dataDxfId="80"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_30세" dataDxfId="79"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_31세" dataDxfId="78"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_32세" dataDxfId="77"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0000-000032000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_33세" dataDxfId="76"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0000-000033000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_34세" dataDxfId="75"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0000-000034000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_35세" dataDxfId="74"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0000-000035000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_36세" dataDxfId="73"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0000-000036000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_37세" dataDxfId="72"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0000-000037000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_38세" dataDxfId="71"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0000-000038000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_39세" dataDxfId="70"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0000-000039000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_40세" dataDxfId="69"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0000-00003A000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_41세" dataDxfId="68"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0000-00003B000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_42세" dataDxfId="67"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0000-00003C000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_43세" dataDxfId="66"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0000-00003D000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_44세" dataDxfId="65"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0000-00003E000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_45세" dataDxfId="64"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0000-00003F000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_46세" dataDxfId="63"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0000-000040000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_47세" dataDxfId="62"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0000-000041000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_48세" dataDxfId="61"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0000-000042000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_49세" dataDxfId="60"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0000-000043000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_50세" dataDxfId="59"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0000-000044000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_51세" dataDxfId="58"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0000-000045000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_52세" dataDxfId="57"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0000-000046000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_53세" dataDxfId="56"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0000-000047000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_54세" dataDxfId="55"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0000-000048000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_55세" dataDxfId="54"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0000-000049000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_56세" dataDxfId="53"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0000-00004A000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_57세" dataDxfId="52"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0000-00004B000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_58세" dataDxfId="51"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0000-00004C000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_59세" dataDxfId="50"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0000-00004D000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_60세" dataDxfId="49"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0000-00004E000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_61세" dataDxfId="48"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0000-00004F000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_62세" dataDxfId="47"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0000-000050000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_63세" dataDxfId="46"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0000-000051000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_64세" dataDxfId="45"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0000-000052000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_65세" dataDxfId="44"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0000-000053000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_66세" dataDxfId="43"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0000-000054000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_67세" dataDxfId="42"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0000-000055000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_68세" dataDxfId="41"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0000-000056000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_69세" dataDxfId="40"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0000-000057000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_70세" dataDxfId="39"/>
+    <tableColumn id="88" xr3:uid="{00000000-0010-0000-0000-000058000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_71세" dataDxfId="38"/>
+    <tableColumn id="89" xr3:uid="{00000000-0010-0000-0000-000059000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_72세" dataDxfId="37"/>
+    <tableColumn id="90" xr3:uid="{00000000-0010-0000-0000-00005A000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_73세" dataDxfId="36"/>
+    <tableColumn id="91" xr3:uid="{00000000-0010-0000-0000-00005B000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_74세" dataDxfId="35"/>
+    <tableColumn id="92" xr3:uid="{00000000-0010-0000-0000-00005C000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_75세" dataDxfId="34"/>
+    <tableColumn id="93" xr3:uid="{00000000-0010-0000-0000-00005D000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_76세" dataDxfId="33"/>
+    <tableColumn id="94" xr3:uid="{00000000-0010-0000-0000-00005E000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_77세" dataDxfId="32"/>
+    <tableColumn id="95" xr3:uid="{00000000-0010-0000-0000-00005F000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_78세" dataDxfId="31"/>
+    <tableColumn id="96" xr3:uid="{00000000-0010-0000-0000-000060000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_79세" dataDxfId="30"/>
+    <tableColumn id="97" xr3:uid="{00000000-0010-0000-0000-000061000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_80세" dataDxfId="29"/>
+    <tableColumn id="98" xr3:uid="{00000000-0010-0000-0000-000062000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_81세" dataDxfId="28"/>
+    <tableColumn id="99" xr3:uid="{00000000-0010-0000-0000-000063000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_82세" dataDxfId="27"/>
+    <tableColumn id="100" xr3:uid="{00000000-0010-0000-0000-000064000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_83세" dataDxfId="26"/>
+    <tableColumn id="101" xr3:uid="{00000000-0010-0000-0000-000065000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_84세" dataDxfId="25"/>
+    <tableColumn id="102" xr3:uid="{00000000-0010-0000-0000-000066000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_85세" dataDxfId="24"/>
+    <tableColumn id="103" xr3:uid="{00000000-0010-0000-0000-000067000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_86세" dataDxfId="23"/>
+    <tableColumn id="104" xr3:uid="{00000000-0010-0000-0000-000068000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_87세" dataDxfId="22"/>
+    <tableColumn id="105" xr3:uid="{00000000-0010-0000-0000-000069000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_88세" dataDxfId="21"/>
+    <tableColumn id="106" xr3:uid="{00000000-0010-0000-0000-00006A000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_89세" dataDxfId="20"/>
+    <tableColumn id="107" xr3:uid="{00000000-0010-0000-0000-00006B000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_90세" dataDxfId="19"/>
+    <tableColumn id="108" xr3:uid="{00000000-0010-0000-0000-00006C000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_91세" dataDxfId="18"/>
+    <tableColumn id="109" xr3:uid="{00000000-0010-0000-0000-00006D000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_92세" dataDxfId="17"/>
+    <tableColumn id="110" xr3:uid="{00000000-0010-0000-0000-00006E000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_93세" dataDxfId="16"/>
+    <tableColumn id="111" xr3:uid="{00000000-0010-0000-0000-00006F000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_94세" dataDxfId="15"/>
+    <tableColumn id="112" xr3:uid="{00000000-0010-0000-0000-000070000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_95세" dataDxfId="14"/>
+    <tableColumn id="113" xr3:uid="{00000000-0010-0000-0000-000071000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_96세" dataDxfId="13"/>
+    <tableColumn id="114" xr3:uid="{00000000-0010-0000-0000-000072000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_97세" dataDxfId="12"/>
+    <tableColumn id="115" xr3:uid="{00000000-0010-0000-0000-000073000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_98세" dataDxfId="11"/>
+    <tableColumn id="116" xr3:uid="{00000000-0010-0000-0000-000074000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_99세" dataDxfId="10"/>
+    <tableColumn id="117" xr3:uid="{00000000-0010-0000-0000-000075000000}" name="행정구역_시군구_별_1세별_주민등록인구(KOSIS 국가통계포털)_2024_총인구수(명)_100세 이상" dataDxfId="9"/>
+    <tableColumn id="118" xr3:uid="{00000000-0010-0000-0000-000076000000}" name="배차간격_요일별(TS 한국교통안전공단)_2024_월_배차간격(분)" dataDxfId="8"/>
+    <tableColumn id="119" xr3:uid="{00000000-0010-0000-0000-000077000000}" name="배차간격_요일별(TS 한국교통안전공단)_2024_화_배차간격(분)" dataDxfId="7"/>
+    <tableColumn id="120" xr3:uid="{00000000-0010-0000-0000-000078000000}" name="배차간격_요일별(TS 한국교통안전공단)_2024_수_배차간격(분)" dataDxfId="6"/>
+    <tableColumn id="121" xr3:uid="{00000000-0010-0000-0000-000079000000}" name="배차간격_요일별(TS 한국교통안전공단)_2024_목_배차간격(분)" dataDxfId="5"/>
+    <tableColumn id="122" xr3:uid="{00000000-0010-0000-0000-00007A000000}" name="배차간격_요일별(TS 한국교통안전공단)_2024_금_배차간격(분)" dataDxfId="4"/>
+    <tableColumn id="123" xr3:uid="{00000000-0010-0000-0000-00007B000000}" name="배차간격_요일별(TS 한국교통안전공단)_2024_토_배차간격(분)" dataDxfId="3"/>
+    <tableColumn id="124" xr3:uid="{00000000-0010-0000-0000-00007C000000}" name="배차간격_요일별(TS 한국교통안전공단)_2024_일_배차간격(분)" dataDxfId="2"/>
+    <tableColumn id="125" xr3:uid="{00000000-0010-0000-0000-00007D000000}" name="시도별_월평균_대중교통비용(KOSIS 국가통계포털)(1)_2024_월평균 비용(만원)" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2354,394 +1375,394 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:DU18"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="125" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:125" ht="110" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="C1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AG1" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AI1" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AJ1" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AL1" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AM1" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AN1" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AO1" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AP1" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AQ1" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AR1" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AS1" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AT1" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AU1" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="2" t="s">
+      <c r="AV1" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="2" t="s">
+      <c r="AW1" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" s="2" t="s">
+      <c r="AX1" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="2" t="s">
+      <c r="AY1" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="AZ1" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="BA1" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BB1" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" s="2" t="s">
+      <c r="BC1" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="2" t="s">
+      <c r="BD1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="2" t="s">
+      <c r="BE1" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" s="2" t="s">
+      <c r="BF1" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" s="2" t="s">
+      <c r="BG1" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" s="2" t="s">
+      <c r="BH1" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" s="2" t="s">
+      <c r="BI1" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" s="2" t="s">
+      <c r="BJ1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" s="2" t="s">
+      <c r="BK1" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" s="2" t="s">
+      <c r="BL1" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" s="2" t="s">
+      <c r="BM1" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="BM1" s="2" t="s">
+      <c r="BN1" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="BN1" s="2" t="s">
+      <c r="BO1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="BO1" s="2" t="s">
+      <c r="BP1" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" s="2" t="s">
+      <c r="BQ1" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="BQ1" s="2" t="s">
+      <c r="BR1" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="BR1" s="2" t="s">
+      <c r="BS1" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="BS1" s="2" t="s">
+      <c r="BT1" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="BT1" s="2" t="s">
+      <c r="BU1" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="BU1" s="2" t="s">
+      <c r="BV1" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="BV1" s="2" t="s">
+      <c r="BW1" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="BW1" s="2" t="s">
+      <c r="BX1" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="BX1" s="2" t="s">
+      <c r="BY1" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="BY1" s="2" t="s">
+      <c r="BZ1" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="BZ1" s="2" t="s">
+      <c r="CA1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="CA1" s="2" t="s">
+      <c r="CB1" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="CB1" s="2" t="s">
+      <c r="CC1" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="CC1" s="2" t="s">
+      <c r="CD1" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="CD1" s="2" t="s">
+      <c r="CE1" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="CE1" s="2" t="s">
+      <c r="CF1" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="CF1" s="2" t="s">
+      <c r="CG1" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="CG1" s="2" t="s">
+      <c r="CH1" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="CH1" s="2" t="s">
+      <c r="CI1" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="CI1" s="2" t="s">
+      <c r="CJ1" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="CJ1" s="2" t="s">
+      <c r="CK1" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="CK1" s="2" t="s">
+      <c r="CL1" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="CL1" s="2" t="s">
+      <c r="CM1" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="CM1" s="2" t="s">
+      <c r="CN1" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="CN1" s="2" t="s">
+      <c r="CO1" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="CO1" s="2" t="s">
+      <c r="CP1" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="CP1" s="2" t="s">
+      <c r="CQ1" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="CQ1" s="2" t="s">
+      <c r="CR1" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="CR1" s="2" t="s">
+      <c r="CS1" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="CS1" s="2" t="s">
+      <c r="CT1" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="CT1" s="2" t="s">
+      <c r="CU1" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="CU1" s="2" t="s">
+      <c r="CV1" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="CV1" s="2" t="s">
+      <c r="CW1" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="CW1" s="2" t="s">
+      <c r="CX1" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="CX1" s="2" t="s">
+      <c r="CY1" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="CY1" s="2" t="s">
+      <c r="CZ1" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="CZ1" s="2" t="s">
+      <c r="DA1" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="DA1" s="2" t="s">
+      <c r="DB1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="DB1" s="2" t="s">
+      <c r="DC1" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="DC1" s="2" t="s">
+      <c r="DD1" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="DD1" s="2" t="s">
+      <c r="DE1" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="DE1" s="2" t="s">
+      <c r="DF1" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="DF1" s="2" t="s">
+      <c r="DG1" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="DG1" s="2" t="s">
+      <c r="DH1" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="DH1" s="2" t="s">
+      <c r="DI1" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="DI1" s="2" t="s">
+      <c r="DJ1" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="DJ1" s="2" t="s">
+      <c r="DK1" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="DK1" s="2" t="s">
+      <c r="DL1" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="DL1" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="DM1" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="DN1" s="2" t="s">
+      <c r="DM1" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="DN1" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="DO1" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="DO1" s="2" t="s">
+      <c r="DP1" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="DP1" s="2" t="s">
+      <c r="DQ1" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="DQ1" s="2" t="s">
+      <c r="DR1" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="DS1" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="DT1" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="DU1" s="17" t="s">
         <v>152</v>
-      </c>
-      <c r="DR1" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="DS1" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="DT1" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="DU1" s="2" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:125" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B2" s="9">
         <v>27.2</v>
@@ -3118,7 +2139,7 @@
     </row>
     <row r="3" spans="1:125" ht="24" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B3" s="13">
         <v>29.8</v>
@@ -3495,7 +2516,7 @@
     </row>
     <row r="4" spans="1:125" ht="24" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B4" s="9">
         <v>30.7</v>
@@ -3873,7 +2894,7 @@
     </row>
     <row r="5" spans="1:125" ht="24" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B5" s="13">
         <v>30.4</v>
@@ -4251,7 +3272,7 @@
     </row>
     <row r="6" spans="1:125" ht="24" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B6" s="9">
         <v>31</v>
@@ -4629,7 +3650,7 @@
     </row>
     <row r="7" spans="1:125" ht="24" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B7" s="13">
         <v>30</v>
@@ -5007,7 +4028,7 @@
     </row>
     <row r="8" spans="1:125" ht="24" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B8" s="9">
         <v>29.8</v>
@@ -5385,7 +4406,7 @@
     </row>
     <row r="9" spans="1:125" ht="24" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B9" s="13">
         <v>35</v>
@@ -5762,7 +4783,7 @@
     </row>
     <row r="10" spans="1:125" ht="24" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B10" s="9">
         <v>31.4</v>
@@ -6140,7 +5161,7 @@
     </row>
     <row r="11" spans="1:125" ht="24" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B11" s="13">
         <v>32.200000000000003</v>
@@ -6517,7 +5538,7 @@
     </row>
     <row r="12" spans="1:125" ht="24" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B12" s="9">
         <v>32.4</v>
@@ -6895,7 +5916,7 @@
     </row>
     <row r="13" spans="1:125" ht="24" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B13" s="13">
         <v>32.700000000000003</v>
@@ -7272,7 +6293,7 @@
     </row>
     <row r="14" spans="1:125" ht="24" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B14" s="9">
         <v>33.1</v>
@@ -7650,7 +6671,7 @@
     </row>
     <row r="15" spans="1:125" ht="24" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B15" s="13">
         <v>33.700000000000003</v>
@@ -8028,7 +7049,7 @@
     </row>
     <row r="16" spans="1:125" ht="24" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B16" s="9">
         <v>32.5</v>
@@ -8406,7 +7427,7 @@
     </row>
     <row r="17" spans="1:125" ht="24" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B17" s="13">
         <v>32.299999999999997</v>
@@ -8784,7 +7805,7 @@
     </row>
     <row r="18" spans="1:125" ht="24" customHeight="1">
       <c r="A18" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B18" s="9">
         <v>29.3</v>
@@ -9170,9 +8191,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="10" width="25" customWidth="1"/>
   </cols>
@@ -9182,36 +8203,36 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
       <c r="A2" s="8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B2" s="8">
         <v>1</v>
@@ -9239,7 +8260,7 @@
     </row>
     <row r="3" spans="1:10" ht="24" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B3" s="5">
         <v>8.6999999999999993</v>
@@ -9273,7 +8294,7 @@
     </row>
     <row r="4" spans="1:10" ht="24" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B4" s="4">
         <v>8.8000000000000007</v>
@@ -9307,7 +8328,7 @@
     </row>
     <row r="5" spans="1:10" ht="24" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B5" s="5">
         <v>8.6999999999999993</v>
@@ -9341,7 +8362,7 @@
     </row>
     <row r="6" spans="1:10" ht="24" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B6" s="4">
         <v>8.4</v>
@@ -9375,7 +8396,7 @@
     </row>
     <row r="7" spans="1:10" ht="24" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B7" s="5">
         <v>7.8</v>
@@ -9409,7 +8430,7 @@
     </row>
     <row r="8" spans="1:10" ht="24" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B8" s="4">
         <v>8.1</v>
@@ -9443,7 +8464,7 @@
     </row>
     <row r="9" spans="1:10" ht="24" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B9" s="5">
         <v>8.1999999999999993</v>
@@ -9477,7 +8498,7 @@
     </row>
     <row r="10" spans="1:10" ht="24" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B10" s="4">
         <v>7.9</v>
@@ -9511,7 +8532,7 @@
     </row>
     <row r="11" spans="1:10" ht="24" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B11" s="5">
         <v>8</v>
@@ -9545,7 +8566,7 @@
     </row>
     <row r="12" spans="1:10" ht="24" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B12" s="4">
         <v>7.8</v>
@@ -9579,7 +8600,7 @@
     </row>
     <row r="13" spans="1:10" ht="24" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B13" s="5">
         <v>6.8</v>
@@ -9613,7 +8634,7 @@
     </row>
     <row r="14" spans="1:10" ht="24" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B14" s="4">
         <v>7.4</v>
@@ -9647,7 +8668,7 @@
     </row>
     <row r="15" spans="1:10" ht="24" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B15" s="5">
         <v>7.6</v>
@@ -9681,7 +8702,7 @@
     </row>
     <row r="16" spans="1:10" ht="24" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B16" s="4">
         <v>7.8</v>
@@ -9715,7 +8736,7 @@
     </row>
     <row r="17" spans="1:10" ht="24" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B17" s="5">
         <v>7.3</v>
@@ -9749,7 +8770,7 @@
     </row>
     <row r="18" spans="1:10" ht="24" customHeight="1">
       <c r="A18" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B18" s="4">
         <v>8</v>
@@ -9783,7 +8804,7 @@
     </row>
     <row r="19" spans="1:10" ht="24" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B19" s="5">
         <v>8.3000000000000007</v>
@@ -9841,7 +8862,7 @@
     </row>
     <row r="22" spans="1:10" ht="24" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -9855,7 +8876,7 @@
     </row>
     <row r="23" spans="1:10" ht="24" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>

</xml_diff>